<commit_message>
Update features and add new files
</commit_message>
<xml_diff>
--- a/backend/sample_leads.xlsx
+++ b/backend/sample_leads.xlsx
@@ -124,6 +124,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>CRM</author>
+  </authors>
+  <commentList>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Enter an RTO code (kl05), office name (Kottayam), or both (KL-05 Kottayam). Close spelling matches are accepted; ambiguous values need review.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -415,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -426,6 +441,7 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -469,6 +485,11 @@
           <t>Enquiry Date</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>RTO</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -977,5 +998,6 @@
   </sheetData>
   <autoFilter ref="A1:H13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>